<commit_message>
Add example-filled edition of the 90-day workbook; Sheets-compatible dropdowns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mn3bcrAxmtz8eaLbtif4v
</commit_message>
<xml_diff>
--- a/youtube_90day/YouTube90日チャレンジ_ワークブック.xlsx
+++ b/youtube_90day/YouTube90日チャレンジ_ワークブック.xlsx
@@ -4967,7 +4967,7 @@
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='03_動画レシピ'!$C$6:$E$6</formula1>
+      <formula1>'03_動画レシピ'!$C$6:$E$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5422,7 +5422,7 @@
       <formula1>"✔"</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='03_動画レシピ'!$C$6:$E$6</formula1>
+      <formula1>'03_動画レシピ'!$C$6:$E$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6350,7 +6350,7 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>レシピ別の平均（自動）</t>
+          <t>レシピ別の平均（スプリント8本・自動）</t>
         </is>
       </c>
       <c r="B18" s="25" t="n"/>
@@ -6412,27 +6412,27 @@
         <v/>
       </c>
       <c r="C20" s="16">
-        <f>IF(B20="","",COUNTIF($C$7:$C$16,B20))</f>
+        <f>IF(B20="","",COUNTIF($C$7:$C$15,B20))</f>
         <v/>
       </c>
       <c r="D20" s="34">
-        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$16,B20,$J$7:$J$16),"-"))</f>
+        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$15,B20,$J$7:$J$15),"-"))</f>
         <v/>
       </c>
       <c r="E20" s="35">
-        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$16,B20,$K$7:$K$16),"-"))</f>
+        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$15,B20,$K$7:$K$15),"-"))</f>
         <v/>
       </c>
       <c r="F20" s="35">
-        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$16,B20,$L$7:$L$16),"-"))</f>
+        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$15,B20,$L$7:$L$15),"-"))</f>
         <v/>
       </c>
       <c r="G20" s="36">
-        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$16,B20,$M$7:$M$16),"-"))</f>
+        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$15,B20,$M$7:$M$15),"-"))</f>
         <v/>
       </c>
       <c r="H20" s="36">
-        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$16,B20,$N$7:$N$16),"-"))</f>
+        <f>IF(B20="","",IFERROR(AVERAGEIF($C$7:$C$15,B20,$N$7:$N$15),"-"))</f>
         <v/>
       </c>
     </row>
@@ -6442,27 +6442,27 @@
         <v/>
       </c>
       <c r="C21" s="16">
-        <f>IF(B21="","",COUNTIF($C$7:$C$16,B21))</f>
+        <f>IF(B21="","",COUNTIF($C$7:$C$15,B21))</f>
         <v/>
       </c>
       <c r="D21" s="34">
-        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$16,B21,$J$7:$J$16),"-"))</f>
+        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$15,B21,$J$7:$J$15),"-"))</f>
         <v/>
       </c>
       <c r="E21" s="35">
-        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$16,B21,$K$7:$K$16),"-"))</f>
+        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$15,B21,$K$7:$K$15),"-"))</f>
         <v/>
       </c>
       <c r="F21" s="35">
-        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$16,B21,$L$7:$L$16),"-"))</f>
+        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$15,B21,$L$7:$L$15),"-"))</f>
         <v/>
       </c>
       <c r="G21" s="36">
-        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$16,B21,$M$7:$M$16),"-"))</f>
+        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$15,B21,$M$7:$M$15),"-"))</f>
         <v/>
       </c>
       <c r="H21" s="36">
-        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$16,B21,$N$7:$N$16),"-"))</f>
+        <f>IF(B21="","",IFERROR(AVERAGEIF($C$7:$C$15,B21,$N$7:$N$15),"-"))</f>
         <v/>
       </c>
     </row>
@@ -6472,34 +6472,34 @@
         <v/>
       </c>
       <c r="C22" s="16">
-        <f>IF(B22="","",COUNTIF($C$7:$C$16,B22))</f>
+        <f>IF(B22="","",COUNTIF($C$7:$C$15,B22))</f>
         <v/>
       </c>
       <c r="D22" s="34">
-        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$16,B22,$J$7:$J$16),"-"))</f>
+        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$15,B22,$J$7:$J$15),"-"))</f>
         <v/>
       </c>
       <c r="E22" s="35">
-        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$16,B22,$K$7:$K$16),"-"))</f>
+        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$15,B22,$K$7:$K$15),"-"))</f>
         <v/>
       </c>
       <c r="F22" s="35">
-        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$16,B22,$L$7:$L$16),"-"))</f>
+        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$15,B22,$L$7:$L$15),"-"))</f>
         <v/>
       </c>
       <c r="G22" s="36">
-        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$16,B22,$M$7:$M$16),"-"))</f>
+        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$15,B22,$M$7:$M$15),"-"))</f>
         <v/>
       </c>
       <c r="H22" s="36">
-        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$16,B22,$N$7:$N$16),"-"))</f>
+        <f>IF(B22="","",IFERROR(AVERAGEIF($C$7:$C$15,B22,$N$7:$N$15),"-"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C7:C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='03_動画レシピ'!$C$6:$E$6</formula1>
+      <formula1>'03_動画レシピ'!$C$6:$E$6</formula1>
     </dataValidation>
     <dataValidation sqref="N7:N16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,5"</formula1>

</xml_diff>

<commit_message>
Split 90-day workbook into prep/production files for Google Drive upload
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mn3bcrAxmtz8eaLbtif4v
</commit_message>
<xml_diff>
--- a/youtube_90day/YouTube90日チャレンジ_ワークブック.xlsx
+++ b/youtube_90day/YouTube90日チャレンジ_ワークブック.xlsx
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="C27" s="17">
-        <f>COUNTA('02_スワイプファイル'!B7:B106)</f>
+        <f>COUNTA('02_スワイプファイル'!B7:B46)</f>
         <v/>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="G4" s="13">
-        <f>COUNTA(B7:B106)&amp;" / 30本"</f>
+        <f>COUNTA(B7:B46)&amp;" / 30本"</f>
         <v/>
       </c>
     </row>
@@ -3257,1035 +3257,15 @@
       <c r="L46" s="21" t="n"/>
       <c r="M46" s="21" t="n"/>
     </row>
-    <row r="47">
-      <c r="A47" s="16" t="n">
-        <v>41</v>
-      </c>
-      <c r="B47" s="21" t="n"/>
-      <c r="C47" s="21" t="n"/>
-      <c r="D47" s="21" t="n"/>
-      <c r="E47" s="21" t="n"/>
-      <c r="F47" s="21" t="n"/>
-      <c r="G47" s="21" t="n"/>
-      <c r="H47" s="21" t="n"/>
-      <c r="I47" s="21" t="n"/>
-      <c r="J47" s="21" t="n"/>
-      <c r="K47" s="21" t="n"/>
-      <c r="L47" s="21" t="n"/>
-      <c r="M47" s="21" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="n">
-        <v>42</v>
-      </c>
-      <c r="B48" s="21" t="n"/>
-      <c r="C48" s="21" t="n"/>
-      <c r="D48" s="21" t="n"/>
-      <c r="E48" s="21" t="n"/>
-      <c r="F48" s="21" t="n"/>
-      <c r="G48" s="21" t="n"/>
-      <c r="H48" s="21" t="n"/>
-      <c r="I48" s="21" t="n"/>
-      <c r="J48" s="21" t="n"/>
-      <c r="K48" s="21" t="n"/>
-      <c r="L48" s="21" t="n"/>
-      <c r="M48" s="21" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="16" t="n">
-        <v>43</v>
-      </c>
-      <c r="B49" s="21" t="n"/>
-      <c r="C49" s="21" t="n"/>
-      <c r="D49" s="21" t="n"/>
-      <c r="E49" s="21" t="n"/>
-      <c r="F49" s="21" t="n"/>
-      <c r="G49" s="21" t="n"/>
-      <c r="H49" s="21" t="n"/>
-      <c r="I49" s="21" t="n"/>
-      <c r="J49" s="21" t="n"/>
-      <c r="K49" s="21" t="n"/>
-      <c r="L49" s="21" t="n"/>
-      <c r="M49" s="21" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="16" t="n">
-        <v>44</v>
-      </c>
-      <c r="B50" s="21" t="n"/>
-      <c r="C50" s="21" t="n"/>
-      <c r="D50" s="21" t="n"/>
-      <c r="E50" s="21" t="n"/>
-      <c r="F50" s="21" t="n"/>
-      <c r="G50" s="21" t="n"/>
-      <c r="H50" s="21" t="n"/>
-      <c r="I50" s="21" t="n"/>
-      <c r="J50" s="21" t="n"/>
-      <c r="K50" s="21" t="n"/>
-      <c r="L50" s="21" t="n"/>
-      <c r="M50" s="21" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="B51" s="21" t="n"/>
-      <c r="C51" s="21" t="n"/>
-      <c r="D51" s="21" t="n"/>
-      <c r="E51" s="21" t="n"/>
-      <c r="F51" s="21" t="n"/>
-      <c r="G51" s="21" t="n"/>
-      <c r="H51" s="21" t="n"/>
-      <c r="I51" s="21" t="n"/>
-      <c r="J51" s="21" t="n"/>
-      <c r="K51" s="21" t="n"/>
-      <c r="L51" s="21" t="n"/>
-      <c r="M51" s="21" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="16" t="n">
-        <v>46</v>
-      </c>
-      <c r="B52" s="21" t="n"/>
-      <c r="C52" s="21" t="n"/>
-      <c r="D52" s="21" t="n"/>
-      <c r="E52" s="21" t="n"/>
-      <c r="F52" s="21" t="n"/>
-      <c r="G52" s="21" t="n"/>
-      <c r="H52" s="21" t="n"/>
-      <c r="I52" s="21" t="n"/>
-      <c r="J52" s="21" t="n"/>
-      <c r="K52" s="21" t="n"/>
-      <c r="L52" s="21" t="n"/>
-      <c r="M52" s="21" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="n">
-        <v>47</v>
-      </c>
-      <c r="B53" s="21" t="n"/>
-      <c r="C53" s="21" t="n"/>
-      <c r="D53" s="21" t="n"/>
-      <c r="E53" s="21" t="n"/>
-      <c r="F53" s="21" t="n"/>
-      <c r="G53" s="21" t="n"/>
-      <c r="H53" s="21" t="n"/>
-      <c r="I53" s="21" t="n"/>
-      <c r="J53" s="21" t="n"/>
-      <c r="K53" s="21" t="n"/>
-      <c r="L53" s="21" t="n"/>
-      <c r="M53" s="21" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="B54" s="21" t="n"/>
-      <c r="C54" s="21" t="n"/>
-      <c r="D54" s="21" t="n"/>
-      <c r="E54" s="21" t="n"/>
-      <c r="F54" s="21" t="n"/>
-      <c r="G54" s="21" t="n"/>
-      <c r="H54" s="21" t="n"/>
-      <c r="I54" s="21" t="n"/>
-      <c r="J54" s="21" t="n"/>
-      <c r="K54" s="21" t="n"/>
-      <c r="L54" s="21" t="n"/>
-      <c r="M54" s="21" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="16" t="n">
-        <v>49</v>
-      </c>
-      <c r="B55" s="21" t="n"/>
-      <c r="C55" s="21" t="n"/>
-      <c r="D55" s="21" t="n"/>
-      <c r="E55" s="21" t="n"/>
-      <c r="F55" s="21" t="n"/>
-      <c r="G55" s="21" t="n"/>
-      <c r="H55" s="21" t="n"/>
-      <c r="I55" s="21" t="n"/>
-      <c r="J55" s="21" t="n"/>
-      <c r="K55" s="21" t="n"/>
-      <c r="L55" s="21" t="n"/>
-      <c r="M55" s="21" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="16" t="n">
-        <v>50</v>
-      </c>
-      <c r="B56" s="21" t="n"/>
-      <c r="C56" s="21" t="n"/>
-      <c r="D56" s="21" t="n"/>
-      <c r="E56" s="21" t="n"/>
-      <c r="F56" s="21" t="n"/>
-      <c r="G56" s="21" t="n"/>
-      <c r="H56" s="21" t="n"/>
-      <c r="I56" s="21" t="n"/>
-      <c r="J56" s="21" t="n"/>
-      <c r="K56" s="21" t="n"/>
-      <c r="L56" s="21" t="n"/>
-      <c r="M56" s="21" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="16" t="n">
-        <v>51</v>
-      </c>
-      <c r="B57" s="21" t="n"/>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="21" t="n"/>
-      <c r="E57" s="21" t="n"/>
-      <c r="F57" s="21" t="n"/>
-      <c r="G57" s="21" t="n"/>
-      <c r="H57" s="21" t="n"/>
-      <c r="I57" s="21" t="n"/>
-      <c r="J57" s="21" t="n"/>
-      <c r="K57" s="21" t="n"/>
-      <c r="L57" s="21" t="n"/>
-      <c r="M57" s="21" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="16" t="n">
-        <v>52</v>
-      </c>
-      <c r="B58" s="21" t="n"/>
-      <c r="C58" s="21" t="n"/>
-      <c r="D58" s="21" t="n"/>
-      <c r="E58" s="21" t="n"/>
-      <c r="F58" s="21" t="n"/>
-      <c r="G58" s="21" t="n"/>
-      <c r="H58" s="21" t="n"/>
-      <c r="I58" s="21" t="n"/>
-      <c r="J58" s="21" t="n"/>
-      <c r="K58" s="21" t="n"/>
-      <c r="L58" s="21" t="n"/>
-      <c r="M58" s="21" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="16" t="n">
-        <v>53</v>
-      </c>
-      <c r="B59" s="21" t="n"/>
-      <c r="C59" s="21" t="n"/>
-      <c r="D59" s="21" t="n"/>
-      <c r="E59" s="21" t="n"/>
-      <c r="F59" s="21" t="n"/>
-      <c r="G59" s="21" t="n"/>
-      <c r="H59" s="21" t="n"/>
-      <c r="I59" s="21" t="n"/>
-      <c r="J59" s="21" t="n"/>
-      <c r="K59" s="21" t="n"/>
-      <c r="L59" s="21" t="n"/>
-      <c r="M59" s="21" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="16" t="n">
-        <v>54</v>
-      </c>
-      <c r="B60" s="21" t="n"/>
-      <c r="C60" s="21" t="n"/>
-      <c r="D60" s="21" t="n"/>
-      <c r="E60" s="21" t="n"/>
-      <c r="F60" s="21" t="n"/>
-      <c r="G60" s="21" t="n"/>
-      <c r="H60" s="21" t="n"/>
-      <c r="I60" s="21" t="n"/>
-      <c r="J60" s="21" t="n"/>
-      <c r="K60" s="21" t="n"/>
-      <c r="L60" s="21" t="n"/>
-      <c r="M60" s="21" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="16" t="n">
-        <v>55</v>
-      </c>
-      <c r="B61" s="21" t="n"/>
-      <c r="C61" s="21" t="n"/>
-      <c r="D61" s="21" t="n"/>
-      <c r="E61" s="21" t="n"/>
-      <c r="F61" s="21" t="n"/>
-      <c r="G61" s="21" t="n"/>
-      <c r="H61" s="21" t="n"/>
-      <c r="I61" s="21" t="n"/>
-      <c r="J61" s="21" t="n"/>
-      <c r="K61" s="21" t="n"/>
-      <c r="L61" s="21" t="n"/>
-      <c r="M61" s="21" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="16" t="n">
-        <v>56</v>
-      </c>
-      <c r="B62" s="21" t="n"/>
-      <c r="C62" s="21" t="n"/>
-      <c r="D62" s="21" t="n"/>
-      <c r="E62" s="21" t="n"/>
-      <c r="F62" s="21" t="n"/>
-      <c r="G62" s="21" t="n"/>
-      <c r="H62" s="21" t="n"/>
-      <c r="I62" s="21" t="n"/>
-      <c r="J62" s="21" t="n"/>
-      <c r="K62" s="21" t="n"/>
-      <c r="L62" s="21" t="n"/>
-      <c r="M62" s="21" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="16" t="n">
-        <v>57</v>
-      </c>
-      <c r="B63" s="21" t="n"/>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
-      <c r="E63" s="21" t="n"/>
-      <c r="F63" s="21" t="n"/>
-      <c r="G63" s="21" t="n"/>
-      <c r="H63" s="21" t="n"/>
-      <c r="I63" s="21" t="n"/>
-      <c r="J63" s="21" t="n"/>
-      <c r="K63" s="21" t="n"/>
-      <c r="L63" s="21" t="n"/>
-      <c r="M63" s="21" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="16" t="n">
-        <v>58</v>
-      </c>
-      <c r="B64" s="21" t="n"/>
-      <c r="C64" s="21" t="n"/>
-      <c r="D64" s="21" t="n"/>
-      <c r="E64" s="21" t="n"/>
-      <c r="F64" s="21" t="n"/>
-      <c r="G64" s="21" t="n"/>
-      <c r="H64" s="21" t="n"/>
-      <c r="I64" s="21" t="n"/>
-      <c r="J64" s="21" t="n"/>
-      <c r="K64" s="21" t="n"/>
-      <c r="L64" s="21" t="n"/>
-      <c r="M64" s="21" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="16" t="n">
-        <v>59</v>
-      </c>
-      <c r="B65" s="21" t="n"/>
-      <c r="C65" s="21" t="n"/>
-      <c r="D65" s="21" t="n"/>
-      <c r="E65" s="21" t="n"/>
-      <c r="F65" s="21" t="n"/>
-      <c r="G65" s="21" t="n"/>
-      <c r="H65" s="21" t="n"/>
-      <c r="I65" s="21" t="n"/>
-      <c r="J65" s="21" t="n"/>
-      <c r="K65" s="21" t="n"/>
-      <c r="L65" s="21" t="n"/>
-      <c r="M65" s="21" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="16" t="n">
-        <v>60</v>
-      </c>
-      <c r="B66" s="21" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
-      <c r="E66" s="21" t="n"/>
-      <c r="F66" s="21" t="n"/>
-      <c r="G66" s="21" t="n"/>
-      <c r="H66" s="21" t="n"/>
-      <c r="I66" s="21" t="n"/>
-      <c r="J66" s="21" t="n"/>
-      <c r="K66" s="21" t="n"/>
-      <c r="L66" s="21" t="n"/>
-      <c r="M66" s="21" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="16" t="n">
-        <v>61</v>
-      </c>
-      <c r="B67" s="21" t="n"/>
-      <c r="C67" s="21" t="n"/>
-      <c r="D67" s="21" t="n"/>
-      <c r="E67" s="21" t="n"/>
-      <c r="F67" s="21" t="n"/>
-      <c r="G67" s="21" t="n"/>
-      <c r="H67" s="21" t="n"/>
-      <c r="I67" s="21" t="n"/>
-      <c r="J67" s="21" t="n"/>
-      <c r="K67" s="21" t="n"/>
-      <c r="L67" s="21" t="n"/>
-      <c r="M67" s="21" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="16" t="n">
-        <v>62</v>
-      </c>
-      <c r="B68" s="21" t="n"/>
-      <c r="C68" s="21" t="n"/>
-      <c r="D68" s="21" t="n"/>
-      <c r="E68" s="21" t="n"/>
-      <c r="F68" s="21" t="n"/>
-      <c r="G68" s="21" t="n"/>
-      <c r="H68" s="21" t="n"/>
-      <c r="I68" s="21" t="n"/>
-      <c r="J68" s="21" t="n"/>
-      <c r="K68" s="21" t="n"/>
-      <c r="L68" s="21" t="n"/>
-      <c r="M68" s="21" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="16" t="n">
-        <v>63</v>
-      </c>
-      <c r="B69" s="21" t="n"/>
-      <c r="C69" s="21" t="n"/>
-      <c r="D69" s="21" t="n"/>
-      <c r="E69" s="21" t="n"/>
-      <c r="F69" s="21" t="n"/>
-      <c r="G69" s="21" t="n"/>
-      <c r="H69" s="21" t="n"/>
-      <c r="I69" s="21" t="n"/>
-      <c r="J69" s="21" t="n"/>
-      <c r="K69" s="21" t="n"/>
-      <c r="L69" s="21" t="n"/>
-      <c r="M69" s="21" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="16" t="n">
-        <v>64</v>
-      </c>
-      <c r="B70" s="21" t="n"/>
-      <c r="C70" s="21" t="n"/>
-      <c r="D70" s="21" t="n"/>
-      <c r="E70" s="21" t="n"/>
-      <c r="F70" s="21" t="n"/>
-      <c r="G70" s="21" t="n"/>
-      <c r="H70" s="21" t="n"/>
-      <c r="I70" s="21" t="n"/>
-      <c r="J70" s="21" t="n"/>
-      <c r="K70" s="21" t="n"/>
-      <c r="L70" s="21" t="n"/>
-      <c r="M70" s="21" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="16" t="n">
-        <v>65</v>
-      </c>
-      <c r="B71" s="21" t="n"/>
-      <c r="C71" s="21" t="n"/>
-      <c r="D71" s="21" t="n"/>
-      <c r="E71" s="21" t="n"/>
-      <c r="F71" s="21" t="n"/>
-      <c r="G71" s="21" t="n"/>
-      <c r="H71" s="21" t="n"/>
-      <c r="I71" s="21" t="n"/>
-      <c r="J71" s="21" t="n"/>
-      <c r="K71" s="21" t="n"/>
-      <c r="L71" s="21" t="n"/>
-      <c r="M71" s="21" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="16" t="n">
-        <v>66</v>
-      </c>
-      <c r="B72" s="21" t="n"/>
-      <c r="C72" s="21" t="n"/>
-      <c r="D72" s="21" t="n"/>
-      <c r="E72" s="21" t="n"/>
-      <c r="F72" s="21" t="n"/>
-      <c r="G72" s="21" t="n"/>
-      <c r="H72" s="21" t="n"/>
-      <c r="I72" s="21" t="n"/>
-      <c r="J72" s="21" t="n"/>
-      <c r="K72" s="21" t="n"/>
-      <c r="L72" s="21" t="n"/>
-      <c r="M72" s="21" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="16" t="n">
-        <v>67</v>
-      </c>
-      <c r="B73" s="21" t="n"/>
-      <c r="C73" s="21" t="n"/>
-      <c r="D73" s="21" t="n"/>
-      <c r="E73" s="21" t="n"/>
-      <c r="F73" s="21" t="n"/>
-      <c r="G73" s="21" t="n"/>
-      <c r="H73" s="21" t="n"/>
-      <c r="I73" s="21" t="n"/>
-      <c r="J73" s="21" t="n"/>
-      <c r="K73" s="21" t="n"/>
-      <c r="L73" s="21" t="n"/>
-      <c r="M73" s="21" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="16" t="n">
-        <v>68</v>
-      </c>
-      <c r="B74" s="21" t="n"/>
-      <c r="C74" s="21" t="n"/>
-      <c r="D74" s="21" t="n"/>
-      <c r="E74" s="21" t="n"/>
-      <c r="F74" s="21" t="n"/>
-      <c r="G74" s="21" t="n"/>
-      <c r="H74" s="21" t="n"/>
-      <c r="I74" s="21" t="n"/>
-      <c r="J74" s="21" t="n"/>
-      <c r="K74" s="21" t="n"/>
-      <c r="L74" s="21" t="n"/>
-      <c r="M74" s="21" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="16" t="n">
-        <v>69</v>
-      </c>
-      <c r="B75" s="21" t="n"/>
-      <c r="C75" s="21" t="n"/>
-      <c r="D75" s="21" t="n"/>
-      <c r="E75" s="21" t="n"/>
-      <c r="F75" s="21" t="n"/>
-      <c r="G75" s="21" t="n"/>
-      <c r="H75" s="21" t="n"/>
-      <c r="I75" s="21" t="n"/>
-      <c r="J75" s="21" t="n"/>
-      <c r="K75" s="21" t="n"/>
-      <c r="L75" s="21" t="n"/>
-      <c r="M75" s="21" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="B76" s="21" t="n"/>
-      <c r="C76" s="21" t="n"/>
-      <c r="D76" s="21" t="n"/>
-      <c r="E76" s="21" t="n"/>
-      <c r="F76" s="21" t="n"/>
-      <c r="G76" s="21" t="n"/>
-      <c r="H76" s="21" t="n"/>
-      <c r="I76" s="21" t="n"/>
-      <c r="J76" s="21" t="n"/>
-      <c r="K76" s="21" t="n"/>
-      <c r="L76" s="21" t="n"/>
-      <c r="M76" s="21" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="16" t="n">
-        <v>71</v>
-      </c>
-      <c r="B77" s="21" t="n"/>
-      <c r="C77" s="21" t="n"/>
-      <c r="D77" s="21" t="n"/>
-      <c r="E77" s="21" t="n"/>
-      <c r="F77" s="21" t="n"/>
-      <c r="G77" s="21" t="n"/>
-      <c r="H77" s="21" t="n"/>
-      <c r="I77" s="21" t="n"/>
-      <c r="J77" s="21" t="n"/>
-      <c r="K77" s="21" t="n"/>
-      <c r="L77" s="21" t="n"/>
-      <c r="M77" s="21" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="16" t="n">
-        <v>72</v>
-      </c>
-      <c r="B78" s="21" t="n"/>
-      <c r="C78" s="21" t="n"/>
-      <c r="D78" s="21" t="n"/>
-      <c r="E78" s="21" t="n"/>
-      <c r="F78" s="21" t="n"/>
-      <c r="G78" s="21" t="n"/>
-      <c r="H78" s="21" t="n"/>
-      <c r="I78" s="21" t="n"/>
-      <c r="J78" s="21" t="n"/>
-      <c r="K78" s="21" t="n"/>
-      <c r="L78" s="21" t="n"/>
-      <c r="M78" s="21" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="16" t="n">
-        <v>73</v>
-      </c>
-      <c r="B79" s="21" t="n"/>
-      <c r="C79" s="21" t="n"/>
-      <c r="D79" s="21" t="n"/>
-      <c r="E79" s="21" t="n"/>
-      <c r="F79" s="21" t="n"/>
-      <c r="G79" s="21" t="n"/>
-      <c r="H79" s="21" t="n"/>
-      <c r="I79" s="21" t="n"/>
-      <c r="J79" s="21" t="n"/>
-      <c r="K79" s="21" t="n"/>
-      <c r="L79" s="21" t="n"/>
-      <c r="M79" s="21" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="16" t="n">
-        <v>74</v>
-      </c>
-      <c r="B80" s="21" t="n"/>
-      <c r="C80" s="21" t="n"/>
-      <c r="D80" s="21" t="n"/>
-      <c r="E80" s="21" t="n"/>
-      <c r="F80" s="21" t="n"/>
-      <c r="G80" s="21" t="n"/>
-      <c r="H80" s="21" t="n"/>
-      <c r="I80" s="21" t="n"/>
-      <c r="J80" s="21" t="n"/>
-      <c r="K80" s="21" t="n"/>
-      <c r="L80" s="21" t="n"/>
-      <c r="M80" s="21" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="16" t="n">
-        <v>75</v>
-      </c>
-      <c r="B81" s="21" t="n"/>
-      <c r="C81" s="21" t="n"/>
-      <c r="D81" s="21" t="n"/>
-      <c r="E81" s="21" t="n"/>
-      <c r="F81" s="21" t="n"/>
-      <c r="G81" s="21" t="n"/>
-      <c r="H81" s="21" t="n"/>
-      <c r="I81" s="21" t="n"/>
-      <c r="J81" s="21" t="n"/>
-      <c r="K81" s="21" t="n"/>
-      <c r="L81" s="21" t="n"/>
-      <c r="M81" s="21" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="16" t="n">
-        <v>76</v>
-      </c>
-      <c r="B82" s="21" t="n"/>
-      <c r="C82" s="21" t="n"/>
-      <c r="D82" s="21" t="n"/>
-      <c r="E82" s="21" t="n"/>
-      <c r="F82" s="21" t="n"/>
-      <c r="G82" s="21" t="n"/>
-      <c r="H82" s="21" t="n"/>
-      <c r="I82" s="21" t="n"/>
-      <c r="J82" s="21" t="n"/>
-      <c r="K82" s="21" t="n"/>
-      <c r="L82" s="21" t="n"/>
-      <c r="M82" s="21" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="16" t="n">
-        <v>77</v>
-      </c>
-      <c r="B83" s="21" t="n"/>
-      <c r="C83" s="21" t="n"/>
-      <c r="D83" s="21" t="n"/>
-      <c r="E83" s="21" t="n"/>
-      <c r="F83" s="21" t="n"/>
-      <c r="G83" s="21" t="n"/>
-      <c r="H83" s="21" t="n"/>
-      <c r="I83" s="21" t="n"/>
-      <c r="J83" s="21" t="n"/>
-      <c r="K83" s="21" t="n"/>
-      <c r="L83" s="21" t="n"/>
-      <c r="M83" s="21" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="16" t="n">
-        <v>78</v>
-      </c>
-      <c r="B84" s="21" t="n"/>
-      <c r="C84" s="21" t="n"/>
-      <c r="D84" s="21" t="n"/>
-      <c r="E84" s="21" t="n"/>
-      <c r="F84" s="21" t="n"/>
-      <c r="G84" s="21" t="n"/>
-      <c r="H84" s="21" t="n"/>
-      <c r="I84" s="21" t="n"/>
-      <c r="J84" s="21" t="n"/>
-      <c r="K84" s="21" t="n"/>
-      <c r="L84" s="21" t="n"/>
-      <c r="M84" s="21" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="16" t="n">
-        <v>79</v>
-      </c>
-      <c r="B85" s="21" t="n"/>
-      <c r="C85" s="21" t="n"/>
-      <c r="D85" s="21" t="n"/>
-      <c r="E85" s="21" t="n"/>
-      <c r="F85" s="21" t="n"/>
-      <c r="G85" s="21" t="n"/>
-      <c r="H85" s="21" t="n"/>
-      <c r="I85" s="21" t="n"/>
-      <c r="J85" s="21" t="n"/>
-      <c r="K85" s="21" t="n"/>
-      <c r="L85" s="21" t="n"/>
-      <c r="M85" s="21" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="16" t="n">
-        <v>80</v>
-      </c>
-      <c r="B86" s="21" t="n"/>
-      <c r="C86" s="21" t="n"/>
-      <c r="D86" s="21" t="n"/>
-      <c r="E86" s="21" t="n"/>
-      <c r="F86" s="21" t="n"/>
-      <c r="G86" s="21" t="n"/>
-      <c r="H86" s="21" t="n"/>
-      <c r="I86" s="21" t="n"/>
-      <c r="J86" s="21" t="n"/>
-      <c r="K86" s="21" t="n"/>
-      <c r="L86" s="21" t="n"/>
-      <c r="M86" s="21" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="16" t="n">
-        <v>81</v>
-      </c>
-      <c r="B87" s="21" t="n"/>
-      <c r="C87" s="21" t="n"/>
-      <c r="D87" s="21" t="n"/>
-      <c r="E87" s="21" t="n"/>
-      <c r="F87" s="21" t="n"/>
-      <c r="G87" s="21" t="n"/>
-      <c r="H87" s="21" t="n"/>
-      <c r="I87" s="21" t="n"/>
-      <c r="J87" s="21" t="n"/>
-      <c r="K87" s="21" t="n"/>
-      <c r="L87" s="21" t="n"/>
-      <c r="M87" s="21" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="16" t="n">
-        <v>82</v>
-      </c>
-      <c r="B88" s="21" t="n"/>
-      <c r="C88" s="21" t="n"/>
-      <c r="D88" s="21" t="n"/>
-      <c r="E88" s="21" t="n"/>
-      <c r="F88" s="21" t="n"/>
-      <c r="G88" s="21" t="n"/>
-      <c r="H88" s="21" t="n"/>
-      <c r="I88" s="21" t="n"/>
-      <c r="J88" s="21" t="n"/>
-      <c r="K88" s="21" t="n"/>
-      <c r="L88" s="21" t="n"/>
-      <c r="M88" s="21" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="16" t="n">
-        <v>83</v>
-      </c>
-      <c r="B89" s="21" t="n"/>
-      <c r="C89" s="21" t="n"/>
-      <c r="D89" s="21" t="n"/>
-      <c r="E89" s="21" t="n"/>
-      <c r="F89" s="21" t="n"/>
-      <c r="G89" s="21" t="n"/>
-      <c r="H89" s="21" t="n"/>
-      <c r="I89" s="21" t="n"/>
-      <c r="J89" s="21" t="n"/>
-      <c r="K89" s="21" t="n"/>
-      <c r="L89" s="21" t="n"/>
-      <c r="M89" s="21" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="16" t="n">
-        <v>84</v>
-      </c>
-      <c r="B90" s="21" t="n"/>
-      <c r="C90" s="21" t="n"/>
-      <c r="D90" s="21" t="n"/>
-      <c r="E90" s="21" t="n"/>
-      <c r="F90" s="21" t="n"/>
-      <c r="G90" s="21" t="n"/>
-      <c r="H90" s="21" t="n"/>
-      <c r="I90" s="21" t="n"/>
-      <c r="J90" s="21" t="n"/>
-      <c r="K90" s="21" t="n"/>
-      <c r="L90" s="21" t="n"/>
-      <c r="M90" s="21" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="16" t="n">
-        <v>85</v>
-      </c>
-      <c r="B91" s="21" t="n"/>
-      <c r="C91" s="21" t="n"/>
-      <c r="D91" s="21" t="n"/>
-      <c r="E91" s="21" t="n"/>
-      <c r="F91" s="21" t="n"/>
-      <c r="G91" s="21" t="n"/>
-      <c r="H91" s="21" t="n"/>
-      <c r="I91" s="21" t="n"/>
-      <c r="J91" s="21" t="n"/>
-      <c r="K91" s="21" t="n"/>
-      <c r="L91" s="21" t="n"/>
-      <c r="M91" s="21" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="16" t="n">
-        <v>86</v>
-      </c>
-      <c r="B92" s="21" t="n"/>
-      <c r="C92" s="21" t="n"/>
-      <c r="D92" s="21" t="n"/>
-      <c r="E92" s="21" t="n"/>
-      <c r="F92" s="21" t="n"/>
-      <c r="G92" s="21" t="n"/>
-      <c r="H92" s="21" t="n"/>
-      <c r="I92" s="21" t="n"/>
-      <c r="J92" s="21" t="n"/>
-      <c r="K92" s="21" t="n"/>
-      <c r="L92" s="21" t="n"/>
-      <c r="M92" s="21" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="16" t="n">
-        <v>87</v>
-      </c>
-      <c r="B93" s="21" t="n"/>
-      <c r="C93" s="21" t="n"/>
-      <c r="D93" s="21" t="n"/>
-      <c r="E93" s="21" t="n"/>
-      <c r="F93" s="21" t="n"/>
-      <c r="G93" s="21" t="n"/>
-      <c r="H93" s="21" t="n"/>
-      <c r="I93" s="21" t="n"/>
-      <c r="J93" s="21" t="n"/>
-      <c r="K93" s="21" t="n"/>
-      <c r="L93" s="21" t="n"/>
-      <c r="M93" s="21" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="16" t="n">
-        <v>88</v>
-      </c>
-      <c r="B94" s="21" t="n"/>
-      <c r="C94" s="21" t="n"/>
-      <c r="D94" s="21" t="n"/>
-      <c r="E94" s="21" t="n"/>
-      <c r="F94" s="21" t="n"/>
-      <c r="G94" s="21" t="n"/>
-      <c r="H94" s="21" t="n"/>
-      <c r="I94" s="21" t="n"/>
-      <c r="J94" s="21" t="n"/>
-      <c r="K94" s="21" t="n"/>
-      <c r="L94" s="21" t="n"/>
-      <c r="M94" s="21" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="16" t="n">
-        <v>89</v>
-      </c>
-      <c r="B95" s="21" t="n"/>
-      <c r="C95" s="21" t="n"/>
-      <c r="D95" s="21" t="n"/>
-      <c r="E95" s="21" t="n"/>
-      <c r="F95" s="21" t="n"/>
-      <c r="G95" s="21" t="n"/>
-      <c r="H95" s="21" t="n"/>
-      <c r="I95" s="21" t="n"/>
-      <c r="J95" s="21" t="n"/>
-      <c r="K95" s="21" t="n"/>
-      <c r="L95" s="21" t="n"/>
-      <c r="M95" s="21" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="16" t="n">
-        <v>90</v>
-      </c>
-      <c r="B96" s="21" t="n"/>
-      <c r="C96" s="21" t="n"/>
-      <c r="D96" s="21" t="n"/>
-      <c r="E96" s="21" t="n"/>
-      <c r="F96" s="21" t="n"/>
-      <c r="G96" s="21" t="n"/>
-      <c r="H96" s="21" t="n"/>
-      <c r="I96" s="21" t="n"/>
-      <c r="J96" s="21" t="n"/>
-      <c r="K96" s="21" t="n"/>
-      <c r="L96" s="21" t="n"/>
-      <c r="M96" s="21" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="16" t="n">
-        <v>91</v>
-      </c>
-      <c r="B97" s="21" t="n"/>
-      <c r="C97" s="21" t="n"/>
-      <c r="D97" s="21" t="n"/>
-      <c r="E97" s="21" t="n"/>
-      <c r="F97" s="21" t="n"/>
-      <c r="G97" s="21" t="n"/>
-      <c r="H97" s="21" t="n"/>
-      <c r="I97" s="21" t="n"/>
-      <c r="J97" s="21" t="n"/>
-      <c r="K97" s="21" t="n"/>
-      <c r="L97" s="21" t="n"/>
-      <c r="M97" s="21" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="16" t="n">
-        <v>92</v>
-      </c>
-      <c r="B98" s="21" t="n"/>
-      <c r="C98" s="21" t="n"/>
-      <c r="D98" s="21" t="n"/>
-      <c r="E98" s="21" t="n"/>
-      <c r="F98" s="21" t="n"/>
-      <c r="G98" s="21" t="n"/>
-      <c r="H98" s="21" t="n"/>
-      <c r="I98" s="21" t="n"/>
-      <c r="J98" s="21" t="n"/>
-      <c r="K98" s="21" t="n"/>
-      <c r="L98" s="21" t="n"/>
-      <c r="M98" s="21" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="16" t="n">
-        <v>93</v>
-      </c>
-      <c r="B99" s="21" t="n"/>
-      <c r="C99" s="21" t="n"/>
-      <c r="D99" s="21" t="n"/>
-      <c r="E99" s="21" t="n"/>
-      <c r="F99" s="21" t="n"/>
-      <c r="G99" s="21" t="n"/>
-      <c r="H99" s="21" t="n"/>
-      <c r="I99" s="21" t="n"/>
-      <c r="J99" s="21" t="n"/>
-      <c r="K99" s="21" t="n"/>
-      <c r="L99" s="21" t="n"/>
-      <c r="M99" s="21" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="16" t="n">
-        <v>94</v>
-      </c>
-      <c r="B100" s="21" t="n"/>
-      <c r="C100" s="21" t="n"/>
-      <c r="D100" s="21" t="n"/>
-      <c r="E100" s="21" t="n"/>
-      <c r="F100" s="21" t="n"/>
-      <c r="G100" s="21" t="n"/>
-      <c r="H100" s="21" t="n"/>
-      <c r="I100" s="21" t="n"/>
-      <c r="J100" s="21" t="n"/>
-      <c r="K100" s="21" t="n"/>
-      <c r="L100" s="21" t="n"/>
-      <c r="M100" s="21" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="16" t="n">
-        <v>95</v>
-      </c>
-      <c r="B101" s="21" t="n"/>
-      <c r="C101" s="21" t="n"/>
-      <c r="D101" s="21" t="n"/>
-      <c r="E101" s="21" t="n"/>
-      <c r="F101" s="21" t="n"/>
-      <c r="G101" s="21" t="n"/>
-      <c r="H101" s="21" t="n"/>
-      <c r="I101" s="21" t="n"/>
-      <c r="J101" s="21" t="n"/>
-      <c r="K101" s="21" t="n"/>
-      <c r="L101" s="21" t="n"/>
-      <c r="M101" s="21" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="16" t="n">
-        <v>96</v>
-      </c>
-      <c r="B102" s="21" t="n"/>
-      <c r="C102" s="21" t="n"/>
-      <c r="D102" s="21" t="n"/>
-      <c r="E102" s="21" t="n"/>
-      <c r="F102" s="21" t="n"/>
-      <c r="G102" s="21" t="n"/>
-      <c r="H102" s="21" t="n"/>
-      <c r="I102" s="21" t="n"/>
-      <c r="J102" s="21" t="n"/>
-      <c r="K102" s="21" t="n"/>
-      <c r="L102" s="21" t="n"/>
-      <c r="M102" s="21" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="16" t="n">
-        <v>97</v>
-      </c>
-      <c r="B103" s="21" t="n"/>
-      <c r="C103" s="21" t="n"/>
-      <c r="D103" s="21" t="n"/>
-      <c r="E103" s="21" t="n"/>
-      <c r="F103" s="21" t="n"/>
-      <c r="G103" s="21" t="n"/>
-      <c r="H103" s="21" t="n"/>
-      <c r="I103" s="21" t="n"/>
-      <c r="J103" s="21" t="n"/>
-      <c r="K103" s="21" t="n"/>
-      <c r="L103" s="21" t="n"/>
-      <c r="M103" s="21" t="n"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="16" t="n">
-        <v>98</v>
-      </c>
-      <c r="B104" s="21" t="n"/>
-      <c r="C104" s="21" t="n"/>
-      <c r="D104" s="21" t="n"/>
-      <c r="E104" s="21" t="n"/>
-      <c r="F104" s="21" t="n"/>
-      <c r="G104" s="21" t="n"/>
-      <c r="H104" s="21" t="n"/>
-      <c r="I104" s="21" t="n"/>
-      <c r="J104" s="21" t="n"/>
-      <c r="K104" s="21" t="n"/>
-      <c r="L104" s="21" t="n"/>
-      <c r="M104" s="21" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="16" t="n">
-        <v>99</v>
-      </c>
-      <c r="B105" s="21" t="n"/>
-      <c r="C105" s="21" t="n"/>
-      <c r="D105" s="21" t="n"/>
-      <c r="E105" s="21" t="n"/>
-      <c r="F105" s="21" t="n"/>
-      <c r="G105" s="21" t="n"/>
-      <c r="H105" s="21" t="n"/>
-      <c r="I105" s="21" t="n"/>
-      <c r="J105" s="21" t="n"/>
-      <c r="K105" s="21" t="n"/>
-      <c r="L105" s="21" t="n"/>
-      <c r="M105" s="21" t="n"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="B106" s="21" t="n"/>
-      <c r="C106" s="21" t="n"/>
-      <c r="D106" s="21" t="n"/>
-      <c r="E106" s="21" t="n"/>
-      <c r="F106" s="21" t="n"/>
-      <c r="G106" s="21" t="n"/>
-      <c r="H106" s="21" t="n"/>
-      <c r="I106" s="21" t="n"/>
-      <c r="J106" s="21" t="n"/>
-      <c r="K106" s="21" t="n"/>
-      <c r="L106" s="21" t="n"/>
-      <c r="M106" s="21" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="D7:D106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D7:D46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Vlog,チャレンジ,チュートリアル,解説,分析,リスト/ランキング,ドキュメンタリー,インタビュー,リアクション,ショート,その他"</formula1>
     </dataValidation>
-    <dataValidation sqref="E7:E106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E7:E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ニッチ内,ニッチ外"</formula1>
     </dataValidation>
-    <dataValidation sqref="M7:M106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M7:M46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>